<commit_message>
fix: match product names with images and add Home Decor products
- Add specific product names for Home Decor & Crafts category (24 products)
- Exclude banner images from product generation
- Use image recognition results for Fashion Jewelry naming
- Regenerate site-data.json with accurate product-image matching
</commit_message>
<xml_diff>
--- a/product_list.xlsx
+++ b/product_list.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I191"/>
+  <dimension ref="A1:I179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -594,12 +594,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>银色耳环</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Silver Earrings</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -918,12 +918,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>水晶项链</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Crystal Necklace</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1206,12 +1206,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>金色首饰套装</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Gold Jewelry Set</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -3181,777 +3181,777 @@
     <row r="77">
       <c r="B77" t="inlineStr">
         <is>
-          <t>YW-FJ-076</t>
+          <t>YW-GA-001</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="F77" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="G77" t="n">
-        <v>0.85</v>
+        <v>0.35</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
-          <t>YW-FJ-077</t>
+          <t>YW-GA-002</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>家居装饰</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Home Decor</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>24</v>
+        <v>200</v>
       </c>
       <c r="F78" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G78" t="n">
         <v>0.5</v>
       </c>
-      <c r="G78" t="n">
-        <v>1.5</v>
-      </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>YW-FJ-078</t>
+          <t>YW-GA-003</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>36</v>
+        <v>500</v>
       </c>
       <c r="F79" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G79" t="n">
         <v>0.8</v>
       </c>
-      <c r="G79" t="n">
-        <v>2</v>
-      </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
-          <t>YW-FJ-079</t>
+          <t>YW-GA-004</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>48</v>
+        <v>1000</v>
       </c>
       <c r="F80" t="n">
-        <v>0.2</v>
+        <v>0.08</v>
       </c>
       <c r="G80" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>YW-FJ-080</t>
+          <t>YW-GA-005</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>60</v>
+        <v>2000</v>
       </c>
       <c r="F81" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G81" t="n">
         <v>0.6</v>
       </c>
-      <c r="G81" t="n">
-        <v>1.8</v>
-      </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>YW-FJ-081</t>
+          <t>YW-GA-006</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="F82" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="G82" t="n">
-        <v>0.85</v>
+        <v>0.35</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>YW-FJ-082</t>
+          <t>YW-GA-007</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>24</v>
+        <v>200</v>
       </c>
       <c r="F83" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G83" t="n">
         <v>0.5</v>
       </c>
-      <c r="G83" t="n">
-        <v>1.5</v>
-      </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>YW-FJ-083</t>
+          <t>YW-GA-008</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>家居装饰</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Home Decor</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>36</v>
+        <v>500</v>
       </c>
       <c r="F84" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G84" t="n">
         <v>0.8</v>
       </c>
-      <c r="G84" t="n">
-        <v>2</v>
-      </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t>YW-FJ-084</t>
+          <t>YW-GA-009</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>48</v>
+        <v>1000</v>
       </c>
       <c r="F85" t="n">
-        <v>0.2</v>
+        <v>0.08</v>
       </c>
       <c r="G85" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t>YW-FJ-085</t>
+          <t>YW-GA-010</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>60</v>
+        <v>2000</v>
       </c>
       <c r="F86" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G86" t="n">
         <v>0.6</v>
       </c>
-      <c r="G86" t="n">
-        <v>1.8</v>
-      </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="B87" t="inlineStr">
         <is>
-          <t>YW-FJ-086</t>
+          <t>YW-GA-011</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>家居装饰</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Home Decor</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="F87" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="G87" t="n">
-        <v>0.85</v>
+        <v>0.35</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
-          <t>YW-FJ-087</t>
+          <t>YW-GA-012</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>24</v>
+        <v>200</v>
       </c>
       <c r="F88" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G88" t="n">
         <v>0.5</v>
       </c>
-      <c r="G88" t="n">
-        <v>1.5</v>
-      </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>YW-FJ-088</t>
+          <t>YW-GA-013</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>36</v>
+        <v>500</v>
       </c>
       <c r="F89" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G89" t="n">
         <v>0.8</v>
       </c>
-      <c r="G89" t="n">
-        <v>2</v>
-      </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="B90" t="inlineStr">
         <is>
-          <t>YW-FJ-089</t>
+          <t>YW-GA-014</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>48</v>
+        <v>1000</v>
       </c>
       <c r="F90" t="n">
-        <v>0.2</v>
+        <v>0.08</v>
       </c>
       <c r="G90" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>YW-FJ-090</t>
+          <t>YW-GA-015</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>60</v>
+        <v>2000</v>
       </c>
       <c r="F91" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G91" t="n">
         <v>0.6</v>
       </c>
-      <c r="G91" t="n">
-        <v>1.8</v>
-      </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>YW-FJ-091</t>
+          <t>YW-GA-016</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="F92" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="G92" t="n">
-        <v>0.85</v>
+        <v>0.35</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>YW-FJ-092</t>
+          <t>YW-GA-017</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>24</v>
+        <v>200</v>
       </c>
       <c r="F93" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G93" t="n">
         <v>0.5</v>
       </c>
-      <c r="G93" t="n">
-        <v>1.5</v>
-      </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>YW-FJ-093</t>
+          <t>YW-BA-001</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>链条肩带</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Chain Strap</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="F94" t="n">
-        <v>0.8</v>
+        <v>0.15</v>
       </c>
       <c r="G94" t="n">
-        <v>2</v>
+        <v>0.6</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>YW-FJ-094</t>
+          <t>YW-BA-002</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>包环</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Bag Ring</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F95" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="G95" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>YW-FJ-095</t>
+          <t>YW-BA-003</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>家居装饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Home Decor</t>
+          <t>Bag Accessory</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="F96" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G96" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>YW-FJ-096</t>
+          <t>YW-BA-004</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>链条肩带</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Chain Strap</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>12</v>
+        <v>500</v>
       </c>
       <c r="F97" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G97" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>YW-FJ-097</t>
+          <t>YW-BA-005</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>家居装饰</t>
+          <t>链条肩带</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Home Decor</t>
+          <t>Chain Strap</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>24</v>
+        <v>1000</v>
       </c>
       <c r="F98" t="n">
         <v>0.5</v>
@@ -3961,177 +3961,177 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" t="inlineStr">
         <is>
-          <t>YW-FJ-098</t>
+          <t>YW-BA-006</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>包环</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Bag Ring</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="F99" t="n">
-        <v>0.8</v>
+        <v>0.15</v>
       </c>
       <c r="G99" t="n">
-        <v>2</v>
+        <v>0.6</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>YW-FJ-099</t>
+          <t>YW-BA-007</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>包环</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Bag Ring</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F100" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="G100" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>YW-FJ-100</t>
+          <t>YW-BA-008</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>箱包配件</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Bag Accessory</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="F101" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G101" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>YW-FJ-101</t>
+          <t>YW-BA-009</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>包环</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Bag Ring</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>12</v>
+        <v>500</v>
       </c>
       <c r="F102" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G102" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>YW-FJ-102</t>
+          <t>YW-BA-010</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>包环</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Bag Ring</t>
         </is>
       </c>
       <c r="E103" t="n">
-        <v>24</v>
+        <v>1000</v>
       </c>
       <c r="F103" t="n">
         <v>0.5</v>
@@ -4141,2045 +4141,2045 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>YW-FJ-103</t>
+          <t>YW-BA-011</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>工艺品</t>
+          <t>箱包配件</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Craft Item</t>
+          <t>Bag Accessory</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="F104" t="n">
-        <v>0.8</v>
+        <v>0.15</v>
       </c>
       <c r="G104" t="n">
-        <v>2</v>
+        <v>0.6</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>YW-FJ-104</t>
+          <t>YW-BA-012</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>节日装饰</t>
+          <t>链条肩带</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Festival Decoration</t>
+          <t>Chain Strap</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F105" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="G105" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>YW-FJ-105</t>
+          <t>YW-BA-013</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>节日装饰</t>
+          <t>包环</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Festival Decoration</t>
+          <t>Bag Ring</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="F106" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="G106" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>YW-GA-001</t>
+          <t>YW-BA-014</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>箱包配件</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Bag Accessory</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F107" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="G107" t="n">
-        <v>0.35</v>
+        <v>0.8</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>YW-GA-002</t>
+          <t>YW-BA-015</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>包环</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Bag Ring</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="F108" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="G108" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>YW-GA-003</t>
+          <t>YW-BA-016</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>箱包配件</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Bag Accessory</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="F109" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="G109" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>YW-GA-004</t>
+          <t>YW-BA-017</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>包环</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Bag Ring</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="F110" t="n">
-        <v>0.08</v>
+        <v>0.3</v>
       </c>
       <c r="G110" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>YW-GA-005</t>
+          <t>YW-BA-018</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>包环</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Bag Ring</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>2000</v>
+        <v>200</v>
       </c>
       <c r="F111" t="n">
-        <v>0.15</v>
+        <v>0.4</v>
       </c>
       <c r="G111" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>YW-GA-006</t>
+          <t>YW-BA-019</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>包环</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Bag Ring</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="F112" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="G112" t="n">
-        <v>0.35</v>
+        <v>0.8</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>YW-GA-007</t>
+          <t>YW-HA-001</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>发圈</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Hair Tie</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>200</v>
+        <v>24</v>
       </c>
       <c r="F113" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="G113" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Hair Accessories</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>发饰</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>YW-GA-008</t>
+          <t>YW-HA-002</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>发圈</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Hair Tie</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>500</v>
+        <v>36</v>
       </c>
       <c r="F114" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G114" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Hair Accessories</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>发饰</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>YW-GA-009</t>
+          <t>YW-HA-003</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>发圈</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Hair Tie</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>1000</v>
+        <v>48</v>
       </c>
       <c r="F115" t="n">
-        <v>0.08</v>
+        <v>0.3</v>
       </c>
       <c r="G115" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Hair Accessories</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>发饰</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>YW-GA-010</t>
+          <t>YW-HA-004</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>发圈</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Hair Tie</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>2000</v>
+        <v>60</v>
       </c>
       <c r="F116" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G116" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Hair Accessories</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>发饰</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>YW-GA-011</t>
+          <t>YW-HA-005</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>发圈</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Hair Tie</t>
         </is>
       </c>
       <c r="E117" t="n">
         <v>100</v>
       </c>
       <c r="F117" t="n">
-        <v>0.05</v>
+        <v>0.5</v>
       </c>
       <c r="G117" t="n">
-        <v>0.35</v>
+        <v>1.5</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Hair Accessories</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>发饰</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>YW-GA-012</t>
+          <t>YW-HA-006</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>发圈</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Hair Tie</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>200</v>
+        <v>24</v>
       </c>
       <c r="F118" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="G118" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Hair Accessories</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>发饰</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>YW-GA-013</t>
+          <t>YW-HA-007</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>发圈</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Hair Tie</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>500</v>
+        <v>36</v>
       </c>
       <c r="F119" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G119" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Hair Accessories</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>发饰</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
-          <t>YW-GA-014</t>
+          <t>YW-TG-001</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>1000</v>
+        <v>24</v>
       </c>
       <c r="F120" t="n">
-        <v>0.08</v>
+        <v>0.5</v>
       </c>
       <c r="G120" t="n">
-        <v>0.4</v>
+        <v>2</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="B121" t="inlineStr">
         <is>
-          <t>YW-GA-015</t>
+          <t>YW-TG-002</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>创意礼品</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Novelty Gift</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>2000</v>
+        <v>48</v>
       </c>
       <c r="F121" t="n">
-        <v>0.15</v>
+        <v>0.8</v>
       </c>
       <c r="G121" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
-          <t>YW-GA-016</t>
+          <t>YW-TG-003</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F122" t="n">
-        <v>0.05</v>
+        <v>1</v>
       </c>
       <c r="G122" t="n">
-        <v>0.35</v>
+        <v>4</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="B123" t="inlineStr">
         <is>
-          <t>YW-GA-017</t>
+          <t>YW-TG-004</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>创意礼品</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Novelty Gift</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F123" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="G123" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="B124" t="inlineStr">
         <is>
-          <t>YW-GA-018</t>
+          <t>YW-TG-005</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F124" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="G124" t="n">
-        <v>0.8</v>
+        <v>2.5</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
-          <t>YW-GA-019</t>
+          <t>YW-TG-006</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>创意礼品</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Novelty Gift</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>1000</v>
+        <v>24</v>
       </c>
       <c r="F125" t="n">
-        <v>0.08</v>
+        <v>0.5</v>
       </c>
       <c r="G125" t="n">
-        <v>0.4</v>
+        <v>2</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="B126" t="inlineStr">
         <is>
-          <t>YW-BA-001</t>
+          <t>YW-TG-007</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>链条肩带</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Chain Strap</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F126" t="n">
-        <v>0.15</v>
+        <v>0.8</v>
       </c>
       <c r="G126" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="B127" t="inlineStr">
         <is>
-          <t>YW-BA-002</t>
+          <t>YW-TG-008</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E127" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F127" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="G127" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="B128" t="inlineStr">
         <is>
-          <t>YW-BA-003</t>
+          <t>YW-TG-009</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Bag Accessory</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E128" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F128" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G128" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="B129" t="inlineStr">
         <is>
-          <t>YW-BA-004</t>
+          <t>YW-TG-010</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>链条肩带</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Chain Strap</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F129" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="G129" t="n">
-        <v>0.8</v>
+        <v>2.5</v>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="B130" t="inlineStr">
         <is>
-          <t>YW-BA-005</t>
+          <t>YW-TG-011</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>链条肩带</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Chain Strap</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>1000</v>
+        <v>24</v>
       </c>
       <c r="F130" t="n">
         <v>0.5</v>
       </c>
       <c r="G130" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="B131" t="inlineStr">
         <is>
-          <t>YW-BA-006</t>
+          <t>YW-TG-012</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E131" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F131" t="n">
-        <v>0.15</v>
+        <v>0.8</v>
       </c>
       <c r="G131" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
-          <t>YW-BA-007</t>
+          <t>YW-TG-013</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E132" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F132" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="G132" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="B133" t="inlineStr">
         <is>
-          <t>YW-BA-008</t>
+          <t>YW-TG-014</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>创意礼品</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Bag Accessory</t>
+          <t>Novelty Gift</t>
         </is>
       </c>
       <c r="E133" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F133" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G133" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="B134" t="inlineStr">
         <is>
-          <t>YW-BA-009</t>
+          <t>YW-TG-015</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F134" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="G134" t="n">
-        <v>0.8</v>
+        <v>2.5</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="B135" t="inlineStr">
         <is>
-          <t>YW-BA-010</t>
+          <t>YW-TG-016</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>创意礼品</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Novelty Gift</t>
         </is>
       </c>
       <c r="E135" t="n">
-        <v>1000</v>
+        <v>24</v>
       </c>
       <c r="F135" t="n">
         <v>0.5</v>
       </c>
       <c r="G135" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="B136" t="inlineStr">
         <is>
-          <t>YW-BA-011</t>
+          <t>YW-TG-017</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Bag Accessory</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E136" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F136" t="n">
-        <v>0.15</v>
+        <v>0.8</v>
       </c>
       <c r="G136" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
-          <t>YW-BA-012</t>
+          <t>YW-TG-018</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>链条肩带</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Chain Strap</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E137" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F137" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="G137" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
         <is>
-          <t>YW-BA-013</t>
+          <t>YW-TG-019</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F138" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G138" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="B139" t="inlineStr">
         <is>
-          <t>YW-BA-014</t>
+          <t>YW-TG-020</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Bag Accessory</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F139" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="G139" t="n">
-        <v>0.8</v>
+        <v>2.5</v>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="B140" t="inlineStr">
         <is>
-          <t>YW-BA-015</t>
+          <t>YW-TG-021</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E140" t="n">
-        <v>1000</v>
+        <v>24</v>
       </c>
       <c r="F140" t="n">
         <v>0.5</v>
       </c>
       <c r="G140" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="B141" t="inlineStr">
         <is>
-          <t>YW-BA-016</t>
+          <t>YW-TG-022</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Bag Accessory</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E141" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F141" t="n">
-        <v>0.15</v>
+        <v>0.8</v>
       </c>
       <c r="G141" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="B142" t="inlineStr">
         <is>
-          <t>YW-BA-017</t>
+          <t>YW-TG-023</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E142" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F142" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="G142" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="B143" t="inlineStr">
         <is>
-          <t>YW-BA-018</t>
+          <t>YW-TG-024</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E143" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F143" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G143" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="B144" t="inlineStr">
         <is>
-          <t>YW-BA-019</t>
+          <t>YW-TG-025</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F144" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="G144" t="n">
-        <v>0.8</v>
+        <v>2.5</v>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="B145" t="inlineStr">
         <is>
-          <t>YW-BA-020</t>
+          <t>YW-TG-026</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>1000</v>
+        <v>24</v>
       </c>
       <c r="F145" t="n">
         <v>0.5</v>
       </c>
       <c r="G145" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="B146" t="inlineStr">
         <is>
-          <t>YW-BA-021</t>
+          <t>YW-TG-027</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>包环</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Bag Ring</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F146" t="n">
-        <v>0.15</v>
+        <v>0.8</v>
       </c>
       <c r="G146" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>Bag Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>箱包配件</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="B147" t="inlineStr">
         <is>
-          <t>YW-HA-001</t>
+          <t>YW-TG-028</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>发圈</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Hair Tie</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="F147" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="G147" t="n">
-        <v>0.9</v>
+        <v>4</v>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Hair Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>发饰</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="B148" t="inlineStr">
         <is>
-          <t>YW-HA-002</t>
+          <t>YW-TG-029</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>发圈</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Hair Tie</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>36</v>
+        <v>100</v>
       </c>
       <c r="F148" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G148" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Hair Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>发饰</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="B149" t="inlineStr">
         <is>
-          <t>YW-HA-003</t>
+          <t>YW-TG-030</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>发圈</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Hair Tie</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="F149" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="G149" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>Hair Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>发饰</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="B150" t="inlineStr">
         <is>
-          <t>YW-HA-004</t>
+          <t>YW-TG-031</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>发圈</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Hair Tie</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E150" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="F150" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="G150" t="n">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>Hair Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>发饰</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="B151" t="inlineStr">
         <is>
-          <t>YW-HA-005</t>
+          <t>YW-TG-032</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>发圈</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Hair Tie</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="F151" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="G151" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>Hair Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>发饰</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="B152" t="inlineStr">
         <is>
-          <t>YW-HA-006</t>
+          <t>YW-TG-033</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>发圈</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Hair Tie</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="F152" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="G152" t="n">
-        <v>0.9</v>
+        <v>4</v>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>Hair Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>发饰</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="B153" t="inlineStr">
         <is>
-          <t>YW-HA-007</t>
+          <t>YW-TG-034</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>发圈</t>
+          <t>毛绒玩具</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Hair Tie</t>
+          <t>Plush Toy</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>36</v>
+        <v>100</v>
       </c>
       <c r="F153" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G153" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>Hair Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>发饰</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="B154" t="inlineStr">
         <is>
-          <t>YW-HA-008</t>
+          <t>YW-TG-035</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>彩色发夹</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Colorful Hair Clip</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="F154" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="G154" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>Hair Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>发饰</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="B155" t="inlineStr">
         <is>
-          <t>YW-HA-009</t>
+          <t>YW-TG-036</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>彩色发夹</t>
+          <t>彩色玩具</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Colorful Hair Clip</t>
+          <t>Colorful Toy</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="F155" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="G155" t="n">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Hair Accessories</t>
+          <t>Toys &amp; Gift</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>发饰</t>
+          <t>玩具礼品</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="B156" t="inlineStr">
         <is>
-          <t>YW-TG-001</t>
+          <t>YW-HD-001</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>毛绒玩具</t>
+          <t>树脂摆件</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Plush Toy</t>
+          <t>Resin Figurine</t>
         </is>
       </c>
       <c r="E156" t="n">
         <v>24</v>
       </c>
       <c r="F156" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G156" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="B157" t="inlineStr">
         <is>
-          <t>YW-TG-002</t>
+          <t>YW-HD-002</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>创意礼品</t>
+          <t>亚克力装饰</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Novelty Gift</t>
+          <t>Acrylic Decoration</t>
         </is>
       </c>
       <c r="E157" t="n">
         <v>48</v>
       </c>
       <c r="F157" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="G157" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="B158" t="inlineStr">
         <is>
-          <t>YW-TG-003</t>
+          <t>YW-HD-003</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>彩色玩具</t>
+          <t>水晶装饰品</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Colorful Toy</t>
+          <t>Crystal Ornament</t>
         </is>
       </c>
       <c r="E158" t="n">
         <v>60</v>
       </c>
       <c r="F158" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G158" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="B159" t="inlineStr">
         <is>
-          <t>YW-TG-004</t>
+          <t>YW-HD-004</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>创意礼品</t>
+          <t>木质工艺品</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Novelty Gift</t>
+          <t>Wooden Craft</t>
         </is>
       </c>
       <c r="E159" t="n">
         <v>100</v>
       </c>
       <c r="F159" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G159" t="n">
         <v>1.5</v>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="B160" t="inlineStr">
         <is>
-          <t>YW-TG-005</t>
+          <t>YW-HD-005</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>毛绒玩具</t>
+          <t>金属墙饰</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Plush Toy</t>
+          <t>Metal Wall Art</t>
         </is>
       </c>
       <c r="E160" t="n">
@@ -6193,173 +6193,173 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="B161" t="inlineStr">
         <is>
-          <t>YW-TG-006</t>
+          <t>YW-HD-006</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>创意礼品</t>
+          <t>陶瓷花瓶</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Novelty Gift</t>
+          <t>Ceramic Vase</t>
         </is>
       </c>
       <c r="E161" t="n">
         <v>24</v>
       </c>
       <c r="F161" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G161" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="B162" t="inlineStr">
         <is>
-          <t>YW-TG-007</t>
+          <t>YW-HD-007</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>彩色玩具</t>
+          <t>玻璃烛台</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Colorful Toy</t>
+          <t>Glass Candle Holder</t>
         </is>
       </c>
       <c r="E162" t="n">
         <v>48</v>
       </c>
       <c r="F162" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="G162" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="B163" t="inlineStr">
         <is>
-          <t>YW-TG-008</t>
+          <t>YW-HD-008</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>毛绒玩具</t>
+          <t>布艺花环</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Plush Toy</t>
+          <t>Fabric Garland</t>
         </is>
       </c>
       <c r="E163" t="n">
         <v>60</v>
       </c>
       <c r="F163" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G163" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="B164" t="inlineStr">
         <is>
-          <t>YW-TG-009</t>
+          <t>YW-HD-009</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>毛绒玩具</t>
+          <t>装饰托盘</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Plush Toy</t>
+          <t>Decorative Tray</t>
         </is>
       </c>
       <c r="E164" t="n">
         <v>100</v>
       </c>
       <c r="F164" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G164" t="n">
         <v>1.5</v>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="B165" t="inlineStr">
         <is>
-          <t>YW-TG-010</t>
+          <t>YW-HD-010</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>毛绒玩具</t>
+          <t>餐桌摆件</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Plush Toy</t>
+          <t>Table Centerpiece</t>
         </is>
       </c>
       <c r="E165" t="n">
@@ -6373,173 +6373,173 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="B166" t="inlineStr">
         <is>
-          <t>YW-TG-011</t>
+          <t>YW-HD-011</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>毛绒玩具</t>
+          <t>壁挂装饰</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Plush Toy</t>
+          <t>Wall Hanging</t>
         </is>
       </c>
       <c r="E166" t="n">
         <v>24</v>
       </c>
       <c r="F166" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G166" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="B167" t="inlineStr">
         <is>
-          <t>YW-TG-012</t>
+          <t>YW-HD-012</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>毛绒玩具</t>
+          <t>搁板装饰</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Plush Toy</t>
+          <t>Shelf Decor</t>
         </is>
       </c>
       <c r="E167" t="n">
         <v>48</v>
       </c>
       <c r="F167" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="G167" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="B168" t="inlineStr">
         <is>
-          <t>YW-TG-013</t>
+          <t>YW-HD-013</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>彩色玩具</t>
+          <t>装饰碗</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Colorful Toy</t>
+          <t>Decorative Bowl</t>
         </is>
       </c>
       <c r="E168" t="n">
         <v>60</v>
       </c>
       <c r="F168" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G168" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="B169" t="inlineStr">
         <is>
-          <t>YW-TG-014</t>
+          <t>YW-HD-014</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>创意礼品</t>
+          <t>花园装饰</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Novelty Gift</t>
+          <t>Garden Decoration</t>
         </is>
       </c>
       <c r="E169" t="n">
         <v>100</v>
       </c>
       <c r="F169" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G169" t="n">
         <v>1.5</v>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="B170" t="inlineStr">
         <is>
-          <t>YW-TG-015</t>
+          <t>YW-HD-015</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>彩色玩具</t>
+          <t>季节花环</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Colorful Toy</t>
+          <t>Seasonal Wreath</t>
         </is>
       </c>
       <c r="E170" t="n">
@@ -6553,173 +6553,173 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="B171" t="inlineStr">
         <is>
-          <t>YW-TG-016</t>
+          <t>YW-HD-016</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>创意礼品</t>
+          <t>相框</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Novelty Gift</t>
+          <t>Photo Frame</t>
         </is>
       </c>
       <c r="E171" t="n">
         <v>24</v>
       </c>
       <c r="F171" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G171" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="B172" t="inlineStr">
         <is>
-          <t>YW-TG-017</t>
+          <t>YW-HD-017</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>毛绒玩具</t>
+          <t>首饰收纳</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Plush Toy</t>
+          <t>Jewelry Organizer</t>
         </is>
       </c>
       <c r="E172" t="n">
         <v>48</v>
       </c>
       <c r="F172" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="G172" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="B173" t="inlineStr">
         <is>
-          <t>YW-TG-018</t>
+          <t>YW-HD-018</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>彩色玩具</t>
+          <t>花盆</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Colorful Toy</t>
+          <t>Plant Pot</t>
         </is>
       </c>
       <c r="E173" t="n">
         <v>60</v>
       </c>
       <c r="F173" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G173" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="B174" t="inlineStr">
         <is>
-          <t>YW-TG-019</t>
+          <t>YW-HD-019</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>彩色玩具</t>
+          <t>灯罩</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Colorful Toy</t>
+          <t>Lamp Shade</t>
         </is>
       </c>
       <c r="E174" t="n">
         <v>100</v>
       </c>
       <c r="F174" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G174" t="n">
         <v>1.5</v>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="B175" t="inlineStr">
         <is>
-          <t>YW-TG-020</t>
+          <t>YW-HD-020</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>彩色玩具</t>
+          <t>窗帘绑带</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Colorful Toy</t>
+          <t>Curtain Tieback</t>
         </is>
       </c>
       <c r="E175" t="n">
@@ -6733,588 +6733,156 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="B176" t="inlineStr">
         <is>
-          <t>YW-TG-021</t>
+          <t>YW-HD-021</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>毛绒玩具</t>
+          <t>门饰花环</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Plush Toy</t>
+          <t>Door Wreath</t>
         </is>
       </c>
       <c r="E176" t="n">
         <v>24</v>
       </c>
       <c r="F176" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G176" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="B177" t="inlineStr">
         <is>
-          <t>YW-TG-022</t>
+          <t>YW-HD-022</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>彩色玩具</t>
+          <t>书挡</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Colorful Toy</t>
+          <t>Bookend</t>
         </is>
       </c>
       <c r="E177" t="n">
         <v>48</v>
       </c>
       <c r="F177" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="G177" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="B178" t="inlineStr">
         <is>
-          <t>YW-TG-023</t>
+          <t>YW-HD-023</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>彩色玩具</t>
+          <t>挂钟</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Colorful Toy</t>
+          <t>Wall Clock</t>
         </is>
       </c>
       <c r="E178" t="n">
         <v>60</v>
       </c>
       <c r="F178" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G178" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="B179" t="inlineStr">
         <is>
-          <t>YW-TG-024</t>
+          <t>YW-HD-024</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>彩色玩具</t>
+          <t>镜框</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Colorful Toy</t>
+          <t>Mirror Frame</t>
         </is>
       </c>
       <c r="E179" t="n">
         <v>100</v>
       </c>
       <c r="F179" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G179" t="n">
         <v>1.5</v>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Toys &amp; Gift</t>
+          <t>Home Decor &amp; Crafts</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>YW-TG-025</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>毛绒玩具</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>Plush Toy</t>
-        </is>
-      </c>
-      <c r="E180" t="n">
-        <v>200</v>
-      </c>
-      <c r="F180" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G180" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="H180" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I180" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>YW-TG-026</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>彩色玩具</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>Colorful Toy</t>
-        </is>
-      </c>
-      <c r="E181" t="n">
-        <v>24</v>
-      </c>
-      <c r="F181" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G181" t="n">
-        <v>2</v>
-      </c>
-      <c r="H181" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I181" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>YW-TG-027</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>毛绒玩具</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>Plush Toy</t>
-        </is>
-      </c>
-      <c r="E182" t="n">
-        <v>48</v>
-      </c>
-      <c r="F182" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G182" t="n">
-        <v>3</v>
-      </c>
-      <c r="H182" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I182" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>YW-TG-028</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>毛绒玩具</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>Plush Toy</t>
-        </is>
-      </c>
-      <c r="E183" t="n">
-        <v>60</v>
-      </c>
-      <c r="F183" t="n">
-        <v>1</v>
-      </c>
-      <c r="G183" t="n">
-        <v>4</v>
-      </c>
-      <c r="H183" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I183" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>YW-TG-029</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>毛绒玩具</t>
-        </is>
-      </c>
-      <c r="D184" t="inlineStr">
-        <is>
-          <t>Plush Toy</t>
-        </is>
-      </c>
-      <c r="E184" t="n">
-        <v>100</v>
-      </c>
-      <c r="F184" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G184" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>YW-TG-030</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>彩色玩具</t>
-        </is>
-      </c>
-      <c r="D185" t="inlineStr">
-        <is>
-          <t>Colorful Toy</t>
-        </is>
-      </c>
-      <c r="E185" t="n">
-        <v>200</v>
-      </c>
-      <c r="F185" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G185" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>YW-TG-031</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>毛绒玩具</t>
-        </is>
-      </c>
-      <c r="D186" t="inlineStr">
-        <is>
-          <t>Plush Toy</t>
-        </is>
-      </c>
-      <c r="E186" t="n">
-        <v>24</v>
-      </c>
-      <c r="F186" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G186" t="n">
-        <v>2</v>
-      </c>
-      <c r="H186" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>YW-TG-032</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>毛绒玩具</t>
-        </is>
-      </c>
-      <c r="D187" t="inlineStr">
-        <is>
-          <t>Plush Toy</t>
-        </is>
-      </c>
-      <c r="E187" t="n">
-        <v>48</v>
-      </c>
-      <c r="F187" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G187" t="n">
-        <v>3</v>
-      </c>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I187" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>YW-TG-033</t>
-        </is>
-      </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>彩色玩具</t>
-        </is>
-      </c>
-      <c r="D188" t="inlineStr">
-        <is>
-          <t>Colorful Toy</t>
-        </is>
-      </c>
-      <c r="E188" t="n">
-        <v>60</v>
-      </c>
-      <c r="F188" t="n">
-        <v>1</v>
-      </c>
-      <c r="G188" t="n">
-        <v>4</v>
-      </c>
-      <c r="H188" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I188" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>YW-TG-034</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>毛绒玩具</t>
-        </is>
-      </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>Plush Toy</t>
-        </is>
-      </c>
-      <c r="E189" t="n">
-        <v>100</v>
-      </c>
-      <c r="F189" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G189" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>YW-TG-035</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>彩色玩具</t>
-        </is>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>Colorful Toy</t>
-        </is>
-      </c>
-      <c r="E190" t="n">
-        <v>200</v>
-      </c>
-      <c r="F190" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G190" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>YW-TG-036</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>彩色玩具</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>Colorful Toy</t>
-        </is>
-      </c>
-      <c r="E191" t="n">
-        <v>24</v>
-      </c>
-      <c r="F191" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G191" t="n">
-        <v>2</v>
-      </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>Toys &amp; Gift</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t>玩具礼品</t>
+          <t>家居装饰工艺品</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: product name-image mismatch & product page layout
- Enhanced image recognition to distinguish bags from jewelry
- Bags now correctly identified as "Leather Handbag" with proper images
- Product page: reduced spacing, more compact layout
- Product page: simplified purchase protection section (4 items instead of 8)
- Product page: smaller buttons, rounded-lg instead of rounded-xl
- Product page: reduced padding and margins throughout
- Sidebar: unified icon colors to navy theme
</commit_message>
<xml_diff>
--- a/product_list.xlsx
+++ b/product_list.xlsx
@@ -558,12 +558,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>金色首饰</t>
+          <t>金色吊坠</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Gold Jewelry</t>
+          <t>Gold Pendant</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -594,12 +594,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>银色耳环</t>
+          <t>时尚配饰</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Silver Earrings</t>
+          <t>Fashion Accessory</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -666,12 +666,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>时尚配饰</t>
+          <t>金色吊坠</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Fashion Accessory</t>
+          <t>Gold Pendant</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -702,12 +702,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>金色吊坠</t>
+          <t>银色链条</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Gold Pendant</t>
+          <t>Silver Chain</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -774,12 +774,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>金色吊坠</t>
+          <t>银色吊坠</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Gold Pendant</t>
+          <t>Silver Pendant</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -846,12 +846,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>金色吊坠</t>
+          <t>银色链条</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Gold Pendant</t>
+          <t>Silver Chain</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -882,12 +882,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>金色吊坠</t>
+          <t>银色首饰</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Gold Pendant</t>
+          <t>Silver Jewelry</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -954,12 +954,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>金色吊坠</t>
+          <t>银色吊坠</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Gold Pendant</t>
+          <t>Silver Pendant</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -990,12 +990,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>银色吊坠</t>
+          <t>银色耳钉</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Silver Pendant</t>
+          <t>Silver Stud Earrings</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1026,12 +1026,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>银色链条</t>
+          <t>垂坠耳环</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Silver Chain</t>
+          <t>Drop Earrings</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1062,12 +1062,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>银色链条</t>
+          <t>戒指</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Silver Chain</t>
+          <t>Ring</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1098,12 +1098,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>金色首饰</t>
+          <t>银色手链</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Gold Jewelry</t>
+          <t>Silver Bracelet</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1134,12 +1134,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>银色首饰</t>
+          <t>金色耳环</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Silver Jewelry</t>
+          <t>Gold Earrings</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1170,12 +1170,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>银色首饰</t>
+          <t>戒指</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Silver Jewelry</t>
+          <t>Ring</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1206,12 +1206,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>金色首饰套装</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Gold Jewelry Set</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1242,12 +1242,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>银色吊坠</t>
+          <t>金色耳钉</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Silver Pendant</t>
+          <t>Gold Stud Earrings</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1278,12 +1278,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>银色耳钉</t>
+          <t>金色耳钉</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Silver Stud Earrings</t>
+          <t>Gold Stud Earrings</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1314,12 +1314,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>垂坠耳环</t>
+          <t>金色耳环</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Drop Earrings</t>
+          <t>Gold Earrings</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>戒指</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Ring</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1386,12 +1386,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>银色手链</t>
+          <t>耳钉</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Silver Bracelet</t>
+          <t>Stud Earrings</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1422,12 +1422,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>金色耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Gold Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1458,12 +1458,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>戒指</t>
+          <t>银色链条手链</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Ring</t>
+          <t>Silver Chain Bracelet</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1494,12 +1494,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>戒指</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Ring</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1530,12 +1530,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>金色耳钉</t>
+          <t>银色戒指</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Gold Stud Earrings</t>
+          <t>Silver Ring</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -1566,12 +1566,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>金色耳钉</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Gold Stud Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -1602,12 +1602,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>金色耳环</t>
+          <t>银色链条手链</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Gold Earrings</t>
+          <t>Silver Chain Bracelet</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色戒指</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Ring</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -1674,12 +1674,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>耳钉</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Stud Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>圆环耳环</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Hoop Earrings</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -1746,12 +1746,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>银色链条手链</t>
+          <t>金色耳钉</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Silver Chain Bracelet</t>
+          <t>Gold Stud Earrings</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -1782,12 +1782,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>戒指</t>
+          <t>银色戒指</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Ring</t>
+          <t>Silver Ring</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -1818,12 +1818,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>银色戒指</t>
+          <t>银色耳钉</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Silver Ring</t>
+          <t>Silver Stud Earrings</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -1854,12 +1854,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>银色戒指</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Silver Ring</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -1890,12 +1890,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>银色链条手链</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Silver Chain Bracelet</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -1926,12 +1926,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>银色戒指</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Silver Ring</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -1962,12 +1962,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>金色耳环</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Gold Earrings</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -1998,12 +1998,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>圆环耳环</t>
+          <t>耳环</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Hoop Earrings</t>
+          <t>Earrings</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -2034,12 +2034,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>金色耳钉</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Gold Stud Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -2070,12 +2070,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>银色戒指</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Silver Ring</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -2106,12 +2106,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>银色耳钉</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Silver Stud Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -2142,12 +2142,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>银色戒指</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Silver Ring</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -2178,12 +2178,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>链条手链</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Chain Bracelet</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -2214,12 +2214,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -2286,12 +2286,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -2322,12 +2322,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>戒指</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Ring</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -2394,12 +2394,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -2430,12 +2430,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -2466,12 +2466,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>链条手链</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Chain Bracelet</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -2502,12 +2502,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -2538,12 +2538,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>金色耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Gold Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -2574,12 +2574,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -2610,12 +2610,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>戒指</t>
+          <t>银色耳钉</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Ring</t>
+          <t>Silver Stud Earrings</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -2646,12 +2646,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>圆环耳环</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Hoop Earrings</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -2718,12 +2718,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色手链</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Bracelet</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -2790,12 +2790,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>圆环耳环</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Hoop Earrings</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -2893,315 +2893,315 @@
     <row r="69">
       <c r="B69" t="inlineStr">
         <is>
-          <t>YW-FJ-068</t>
+          <t>YW-GA-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>银色耳钉</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Silver Stud Earrings</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>36</v>
+        <v>100</v>
       </c>
       <c r="F69" t="n">
-        <v>0.8</v>
+        <v>0.05</v>
       </c>
       <c r="G69" t="n">
-        <v>2</v>
+        <v>0.35</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" t="inlineStr">
         <is>
-          <t>YW-FJ-069</t>
+          <t>YW-GA-002</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>圆环耳环</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Hoop Earrings</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="F70" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G70" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" t="inlineStr">
         <is>
-          <t>YW-FJ-070</t>
+          <t>YW-GA-003</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>60</v>
+        <v>500</v>
       </c>
       <c r="F71" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="G71" t="n">
-        <v>1.8</v>
+        <v>0.8</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
-          <t>YW-FJ-071</t>
+          <t>YW-GA-004</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>银色手链</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Silver Bracelet</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>12</v>
+        <v>1000</v>
       </c>
       <c r="F72" t="n">
-        <v>0.15</v>
+        <v>0.08</v>
       </c>
       <c r="G72" t="n">
-        <v>0.85</v>
+        <v>0.4</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" t="inlineStr">
         <is>
-          <t>YW-FJ-072</t>
+          <t>YW-GA-005</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>24</v>
+        <v>2000</v>
       </c>
       <c r="F73" t="n">
-        <v>0.5</v>
+        <v>0.15</v>
       </c>
       <c r="G73" t="n">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
-          <t>YW-FJ-073</t>
+          <t>YW-GA-006</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>圆环耳环</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Hoop Earrings</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>36</v>
+        <v>100</v>
       </c>
       <c r="F74" t="n">
-        <v>0.8</v>
+        <v>0.05</v>
       </c>
       <c r="G74" t="n">
-        <v>2</v>
+        <v>0.35</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
         <is>
-          <t>YW-FJ-074</t>
+          <t>YW-GA-007</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="F75" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G75" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" t="inlineStr">
         <is>
-          <t>YW-FJ-075</t>
+          <t>YW-GA-008</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>60</v>
+        <v>500</v>
       </c>
       <c r="F76" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="G76" t="n">
-        <v>1.8</v>
+        <v>0.8</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" t="inlineStr">
         <is>
-          <t>YW-GA-001</t>
+          <t>YW-GA-009</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="F77" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="G77" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -3217,7 +3217,7 @@
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
-          <t>YW-GA-002</t>
+          <t>YW-GA-010</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3231,13 +3231,13 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>200</v>
+        <v>2000</v>
       </c>
       <c r="F78" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="G78" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -3253,27 +3253,27 @@
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>YW-GA-003</t>
+          <t>YW-GA-011</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F79" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="G79" t="n">
-        <v>0.8</v>
+        <v>0.35</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -3289,27 +3289,27 @@
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
-          <t>YW-GA-004</t>
+          <t>YW-GA-012</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="F80" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="G80" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -3325,27 +3325,27 @@
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>YW-GA-005</t>
+          <t>YW-GA-013</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="F81" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G81" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -3361,27 +3361,27 @@
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>YW-GA-006</t>
+          <t>YW-GA-014</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="F82" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="G82" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -3397,7 +3397,7 @@
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>YW-GA-007</t>
+          <t>YW-GA-015</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3411,13 +3411,13 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>200</v>
+        <v>2000</v>
       </c>
       <c r="F83" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="G83" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>YW-GA-008</t>
+          <t>YW-GA-016</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3447,13 +3447,13 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F84" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="G84" t="n">
-        <v>0.8</v>
+        <v>0.35</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -3469,27 +3469,27 @@
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t>YW-GA-009</t>
+          <t>YW-GA-017</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="F85" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="G85" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -3505,21 +3505,21 @@
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t>YW-GA-010</t>
+          <t>YW-BA-001</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>2000</v>
+        <v>50</v>
       </c>
       <c r="F86" t="n">
         <v>0.15</v>
@@ -3529,101 +3529,101 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="B87" t="inlineStr">
         <is>
-          <t>YW-GA-011</t>
+          <t>YW-BA-002</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E87" t="n">
         <v>100</v>
       </c>
       <c r="F87" t="n">
-        <v>0.05</v>
+        <v>0.3</v>
       </c>
       <c r="G87" t="n">
-        <v>0.35</v>
+        <v>1</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
-          <t>YW-GA-012</t>
+          <t>YW-BA-003</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E88" t="n">
         <v>200</v>
       </c>
       <c r="F88" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="G88" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>YW-GA-013</t>
+          <t>YW-BA-004</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -3637,69 +3637,69 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="B90" t="inlineStr">
         <is>
-          <t>YW-GA-014</t>
+          <t>YW-BA-005</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E90" t="n">
         <v>1000</v>
       </c>
       <c r="F90" t="n">
-        <v>0.08</v>
+        <v>0.5</v>
       </c>
       <c r="G90" t="n">
-        <v>0.4</v>
+        <v>1.5</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>YW-GA-015</t>
+          <t>YW-BA-006</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>2000</v>
+        <v>50</v>
       </c>
       <c r="F91" t="n">
         <v>0.15</v>
@@ -3709,91 +3709,91 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>YW-GA-016</t>
+          <t>YW-BA-007</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E92" t="n">
         <v>100</v>
       </c>
       <c r="F92" t="n">
-        <v>0.05</v>
+        <v>0.3</v>
       </c>
       <c r="G92" t="n">
-        <v>0.35</v>
+        <v>1</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>YW-GA-017</t>
+          <t>YW-BA-008</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E93" t="n">
         <v>200</v>
       </c>
       <c r="F93" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="G93" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>YW-BA-001</t>
+          <t>YW-BA-009</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="F94" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G94" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -3829,7 +3829,7 @@
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>YW-BA-002</t>
+          <t>YW-BA-010</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3843,13 +3843,13 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="F95" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="G95" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -3865,7 +3865,7 @@
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>YW-BA-003</t>
+          <t>YW-BA-011</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3879,13 +3879,13 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="F96" t="n">
-        <v>0.4</v>
+        <v>0.15</v>
       </c>
       <c r="G96" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -3901,7 +3901,7 @@
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>YW-BA-004</t>
+          <t>YW-BA-012</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3915,13 +3915,13 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F97" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="G97" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -3937,7 +3937,7 @@
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>YW-BA-005</t>
+          <t>YW-BA-013</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3951,13 +3951,13 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="F98" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G98" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="99">
       <c r="B99" t="inlineStr">
         <is>
-          <t>YW-BA-006</t>
+          <t>YW-BA-014</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3987,13 +3987,13 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="F99" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G99" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -4009,7 +4009,7 @@
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>YW-BA-007</t>
+          <t>YW-BA-015</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4023,13 +4023,13 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="F100" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="G100" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -4045,7 +4045,7 @@
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>YW-BA-008</t>
+          <t>YW-BA-016</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4059,13 +4059,13 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="F101" t="n">
-        <v>0.4</v>
+        <v>0.15</v>
       </c>
       <c r="G101" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -4081,7 +4081,7 @@
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>YW-BA-009</t>
+          <t>YW-BA-017</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4095,13 +4095,13 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F102" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="G102" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -4117,7 +4117,7 @@
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>YW-BA-010</t>
+          <t>YW-BA-018</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4131,13 +4131,13 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="F103" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G103" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -4153,7 +4153,7 @@
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>YW-BA-011</t>
+          <t>YW-BA-019</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4167,13 +4167,13 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="F104" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G104" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -4189,7 +4189,7 @@
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>YW-BA-012</t>
+          <t>YW-BA-020</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4203,13 +4203,13 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="F105" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="G105" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -4225,7 +4225,7 @@
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>YW-BA-013</t>
+          <t>YW-BA-021</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4239,13 +4239,13 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="F106" t="n">
-        <v>0.4</v>
+        <v>0.15</v>
       </c>
       <c r="G106" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -4261,7 +4261,7 @@
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>YW-BA-014</t>
+          <t>YW-BA-022</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4275,13 +4275,13 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F107" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="G107" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -4297,7 +4297,7 @@
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>YW-BA-015</t>
+          <t>YW-BA-023</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -4311,13 +4311,13 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="F108" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G108" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -4333,7 +4333,7 @@
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>YW-BA-016</t>
+          <t>YW-BA-024</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4347,13 +4347,13 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="F109" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G109" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -4369,7 +4369,7 @@
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>YW-BA-017</t>
+          <t>YW-BA-025</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4383,13 +4383,13 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="F110" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="G110" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -4405,7 +4405,7 @@
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>YW-BA-018</t>
+          <t>YW-BA-026</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4419,13 +4419,13 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="F111" t="n">
-        <v>0.4</v>
+        <v>0.15</v>
       </c>
       <c r="G111" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -4441,7 +4441,7 @@
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>YW-BA-019</t>
+          <t>YW-BA-027</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4455,13 +4455,13 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F112" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="G112" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: improve bag image recognition accuracy
- Enhanced bag detection: low edge density + white/silver background = bag
- Fixed white background being misidentified as silver jewelry
- Top Deals now sorted by price (lowest first)
- Bag Accessories category: 36 products with correct names
</commit_message>
<xml_diff>
--- a/product_list.xlsx
+++ b/product_list.xlsx
@@ -486,12 +486,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>银色链条</t>
+          <t>时尚配饰</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Silver Chain</t>
+          <t>Fashion Accessory</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -522,12 +522,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>银色首饰</t>
+          <t>银色链条</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Silver Jewelry</t>
+          <t>Silver Chain</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -558,12 +558,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>金色吊坠</t>
+          <t>银色链条</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Gold Pendant</t>
+          <t>Silver Chain</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -594,12 +594,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>时尚配饰</t>
+          <t>银色链条</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fashion Accessory</t>
+          <t>Silver Chain</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -630,12 +630,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>金色吊坠</t>
+          <t>金色手链</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Gold Pendant</t>
+          <t>Gold Bracelet</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -666,12 +666,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>金色吊坠</t>
+          <t>银色耳钉</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Gold Pendant</t>
+          <t>Silver Stud Earrings</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -702,12 +702,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>银色链条</t>
+          <t>垂坠耳环</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Silver Chain</t>
+          <t>Drop Earrings</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -738,12 +738,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>金色吊坠</t>
+          <t>戒指</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Gold Pendant</t>
+          <t>Ring</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -774,12 +774,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>银色吊坠</t>
+          <t>银色手链</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Silver Pendant</t>
+          <t>Silver Bracelet</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -810,12 +810,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>银色链条</t>
+          <t>金色耳环</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Silver Chain</t>
+          <t>Gold Earrings</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -846,12 +846,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>银色链条</t>
+          <t>戒指</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Silver Chain</t>
+          <t>Ring</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -882,12 +882,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>银色首饰</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Silver Jewelry</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -918,12 +918,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>水晶项链</t>
+          <t>金色耳钉</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Crystal Necklace</t>
+          <t>Gold Stud Earrings</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -954,12 +954,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>银色吊坠</t>
+          <t>金色耳钉</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Silver Pendant</t>
+          <t>Gold Stud Earrings</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -990,12 +990,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>银色耳钉</t>
+          <t>金色耳环</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Silver Stud Earrings</t>
+          <t>Gold Earrings</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1026,12 +1026,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>垂坠耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Drop Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1062,12 +1062,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>戒指</t>
+          <t>耳钉</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Ring</t>
+          <t>Stud Earrings</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1098,12 +1098,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>银色手链</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Silver Bracelet</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1134,12 +1134,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>金色耳环</t>
+          <t>银色链条手链</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Gold Earrings</t>
+          <t>Silver Chain Bracelet</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1206,12 +1206,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>银色戒指</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Silver Ring</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1242,12 +1242,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>金色耳钉</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Gold Stud Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1278,12 +1278,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>金色耳钉</t>
+          <t>银色链条手链</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Gold Stud Earrings</t>
+          <t>Silver Chain Bracelet</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1314,12 +1314,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>金色耳环</t>
+          <t>银色戒指</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Gold Earrings</t>
+          <t>Silver Ring</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1386,12 +1386,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>耳钉</t>
+          <t>圆环耳环</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Stud Earrings</t>
+          <t>Hoop Earrings</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1422,12 +1422,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>金色耳钉</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Gold Stud Earrings</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1458,12 +1458,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>银色链条手链</t>
+          <t>银色戒指</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Silver Chain Bracelet</t>
+          <t>Silver Ring</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1494,12 +1494,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>戒指</t>
+          <t>银色耳钉</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Ring</t>
+          <t>Silver Stud Earrings</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1602,12 +1602,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>银色链条手链</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Silver Chain Bracelet</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>银色戒指</t>
+          <t>金色耳环</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Silver Ring</t>
+          <t>Gold Earrings</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -1674,12 +1674,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>耳环</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Earrings</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>圆环耳环</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Hoop Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -1746,12 +1746,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>金色耳钉</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Gold Stud Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -1782,12 +1782,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>银色戒指</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Silver Ring</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -1818,12 +1818,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>银色耳钉</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Silver Stud Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -1854,12 +1854,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>银色戒指</t>
+          <t>链条手链</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Silver Ring</t>
+          <t>Chain Bracelet</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -1890,12 +1890,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -1926,12 +1926,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>金色耳环</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Gold Earrings</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -1962,12 +1962,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>金色耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Gold Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -1998,12 +1998,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>耳环</t>
+          <t>戒指</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Earrings</t>
+          <t>Ring</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -2034,12 +2034,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -2070,12 +2070,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -2142,12 +2142,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -2178,12 +2178,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>链条手链</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Chain Bracelet</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -2250,12 +2250,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>金色耳环</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Gold Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -2286,12 +2286,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色耳钉</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Stud Earrings</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -2322,12 +2322,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>戒指</t>
+          <t>圆环耳环</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Ring</t>
+          <t>Hoop Earrings</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -2358,12 +2358,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -2394,12 +2394,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>银色手链</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Silver Bracelet</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -2466,12 +2466,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>圆环耳环</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Hoop Earrings</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -2502,12 +2502,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>金色圆环耳环</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Gold Hoop Earrings</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -2538,12 +2538,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色圆环耳环</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Hoop Earrings</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -2569,351 +2569,351 @@
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t>YW-FJ-059</t>
+          <t>YW-GA-001</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F60" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="G60" t="n">
-        <v>0.9</v>
+        <v>0.35</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
         <is>
-          <t>YW-FJ-060</t>
+          <t>YW-GA-002</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>银色耳钉</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Silver Stud Earrings</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="F61" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="G61" t="n">
-        <v>1.8</v>
+        <v>0.5</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
-          <t>YW-FJ-061</t>
+          <t>YW-GA-003</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>圆环耳环</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Hoop Earrings</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>12</v>
+        <v>500</v>
       </c>
       <c r="F62" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G62" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t>YW-FJ-062</t>
+          <t>YW-GA-004</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>24</v>
+        <v>1000</v>
       </c>
       <c r="F63" t="n">
-        <v>0.5</v>
+        <v>0.08</v>
       </c>
       <c r="G63" t="n">
-        <v>1.5</v>
+        <v>0.4</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>YW-FJ-063</t>
+          <t>YW-GA-005</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>银色手链</t>
+          <t>金色纽扣</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Silver Bracelet</t>
+          <t>Gold Button</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>36</v>
+        <v>2000</v>
       </c>
       <c r="F64" t="n">
-        <v>0.8</v>
+        <v>0.15</v>
       </c>
       <c r="G64" t="n">
-        <v>2</v>
+        <v>0.6</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" t="inlineStr">
         <is>
-          <t>YW-FJ-064</t>
+          <t>YW-GA-006</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F65" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="G65" t="n">
-        <v>0.9</v>
+        <v>0.35</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" t="inlineStr">
         <is>
-          <t>YW-FJ-065</t>
+          <t>YW-GA-007</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>圆环耳环</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Hoop Earrings</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="F66" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="G66" t="n">
-        <v>1.8</v>
+        <v>0.5</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="B67" t="inlineStr">
         <is>
-          <t>YW-FJ-066</t>
+          <t>YW-GA-008</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>金色圆环耳环</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Gold Hoop Earrings</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>12</v>
+        <v>500</v>
       </c>
       <c r="F67" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G67" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" t="inlineStr">
         <is>
-          <t>YW-FJ-067</t>
+          <t>YW-GA-009</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>银色圆环耳环</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Silver Hoop Earrings</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>24</v>
+        <v>1000</v>
       </c>
       <c r="F68" t="n">
-        <v>0.5</v>
+        <v>0.08</v>
       </c>
       <c r="G68" t="n">
-        <v>1.5</v>
+        <v>0.4</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Fashion Jewelry</t>
+          <t>Garment Accessories</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>时尚首饰</t>
+          <t>服装辅料</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="B69" t="inlineStr">
         <is>
-          <t>YW-GA-001</t>
+          <t>YW-GA-010</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>100</v>
+        <v>2000</v>
       </c>
       <c r="F69" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="G69" t="n">
-        <v>0.35</v>
+        <v>0.6</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -2929,27 +2929,27 @@
     <row r="70">
       <c r="B70" t="inlineStr">
         <is>
-          <t>YW-GA-002</t>
+          <t>YW-GA-011</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F70" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G70" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -2965,7 +2965,7 @@
     <row r="71">
       <c r="B71" t="inlineStr">
         <is>
-          <t>YW-GA-003</t>
+          <t>YW-GA-012</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2979,13 +2979,13 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F71" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G71" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -3001,27 +3001,27 @@
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
-          <t>YW-GA-004</t>
+          <t>YW-GA-013</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F72" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="G72" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -3037,7 +3037,7 @@
     <row r="73">
       <c r="B73" t="inlineStr">
         <is>
-          <t>YW-GA-005</t>
+          <t>YW-GA-014</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3051,13 +3051,13 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F73" t="n">
-        <v>0.15</v>
+        <v>0.08</v>
       </c>
       <c r="G73" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -3073,27 +3073,27 @@
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
-          <t>YW-GA-006</t>
+          <t>YW-GA-015</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>服装配件</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Garment Accessory</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>100</v>
+        <v>2000</v>
       </c>
       <c r="F74" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="G74" t="n">
-        <v>0.35</v>
+        <v>0.6</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -3109,7 +3109,7 @@
     <row r="75">
       <c r="B75" t="inlineStr">
         <is>
-          <t>YW-GA-007</t>
+          <t>YW-GA-016</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3123,13 +3123,13 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F75" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G75" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -3145,27 +3145,27 @@
     <row r="76">
       <c r="B76" t="inlineStr">
         <is>
-          <t>YW-GA-008</t>
+          <t>YW-GA-017</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>银色纽扣</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Silver Button</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F76" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G76" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -3181,351 +3181,351 @@
     <row r="77">
       <c r="B77" t="inlineStr">
         <is>
-          <t>YW-GA-009</t>
+          <t>YW-BA-001</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>1000</v>
+        <v>50</v>
       </c>
       <c r="F77" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="G77" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
-          <t>YW-GA-010</t>
+          <t>YW-BA-002</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>2000</v>
+        <v>100</v>
       </c>
       <c r="F78" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="G78" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>YW-GA-011</t>
+          <t>YW-BA-003</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F79" t="n">
-        <v>0.05</v>
+        <v>0.4</v>
       </c>
       <c r="G79" t="n">
-        <v>0.35</v>
+        <v>1.2</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
-          <t>YW-GA-012</t>
+          <t>YW-BA-004</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="F80" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G80" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>YW-GA-013</t>
+          <t>YW-BA-005</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>时尚手提包</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Fashion Handbag</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="F81" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="G81" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>YW-GA-014</t>
+          <t>YW-BA-006</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>金色纽扣</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Gold Button</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>1000</v>
+        <v>50</v>
       </c>
       <c r="F82" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="G82" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>YW-GA-015</t>
+          <t>YW-BA-007</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>时尚手提包</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Fashion Handbag</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>2000</v>
+        <v>100</v>
       </c>
       <c r="F83" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="G83" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>YW-GA-016</t>
+          <t>YW-BA-008</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>服装配件</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Garment Accessory</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F84" t="n">
-        <v>0.05</v>
+        <v>0.4</v>
       </c>
       <c r="G84" t="n">
-        <v>0.35</v>
+        <v>1.2</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t>YW-GA-017</t>
+          <t>YW-BA-009</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>银色纽扣</t>
+          <t>皮革手提包</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Silver Button</t>
+          <t>Leather Handbag</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="F85" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G85" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Garment Accessories</t>
+          <t>Bag Accessories</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>服装辅料</t>
+          <t>箱包配件</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t>YW-BA-001</t>
+          <t>YW-BA-010</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>皮革手提包</t>
+          <t>时尚手提包</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Leather Handbag</t>
+          <t>Fashion Handbag</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="F86" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="G86" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -3541,7 +3541,7 @@
     <row r="87">
       <c r="B87" t="inlineStr">
         <is>
-          <t>YW-BA-002</t>
+          <t>YW-BA-011</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3555,13 +3555,13 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F87" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G87" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -3577,7 +3577,7 @@
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
-          <t>YW-BA-003</t>
+          <t>YW-BA-012</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3591,13 +3591,13 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F88" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G88" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -3613,7 +3613,7 @@
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>YW-BA-004</t>
+          <t>YW-BA-013</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3627,13 +3627,13 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F89" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G89" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -3649,7 +3649,7 @@
     <row r="90">
       <c r="B90" t="inlineStr">
         <is>
-          <t>YW-BA-005</t>
+          <t>YW-BA-014</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3663,13 +3663,13 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F90" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="G90" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -3685,7 +3685,7 @@
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>YW-BA-006</t>
+          <t>YW-BA-015</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3699,13 +3699,13 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="F91" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="G91" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -3721,7 +3721,7 @@
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>YW-BA-007</t>
+          <t>YW-BA-016</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3735,13 +3735,13 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F92" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G92" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -3757,7 +3757,7 @@
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>YW-BA-008</t>
+          <t>YW-BA-017</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3771,13 +3771,13 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F93" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G93" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -3793,7 +3793,7 @@
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>YW-BA-009</t>
+          <t>YW-BA-018</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F94" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G94" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -3829,7 +3829,7 @@
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>YW-BA-010</t>
+          <t>YW-BA-019</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3843,13 +3843,13 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F95" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="G95" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
@@ -3865,7 +3865,7 @@
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>YW-BA-011</t>
+          <t>YW-BA-020</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3879,13 +3879,13 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="F96" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="G96" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -3901,7 +3901,7 @@
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>YW-BA-012</t>
+          <t>YW-BA-021</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3915,13 +3915,13 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F97" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G97" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -3937,7 +3937,7 @@
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>YW-BA-013</t>
+          <t>YW-BA-022</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3951,13 +3951,13 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F98" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G98" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="99">
       <c r="B99" t="inlineStr">
         <is>
-          <t>YW-BA-014</t>
+          <t>YW-BA-023</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3987,13 +3987,13 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F99" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G99" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -4009,7 +4009,7 @@
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>YW-BA-015</t>
+          <t>YW-BA-024</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4023,13 +4023,13 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F100" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="G100" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -4045,7 +4045,7 @@
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>YW-BA-016</t>
+          <t>YW-BA-025</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4059,13 +4059,13 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="F101" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="G101" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -4081,7 +4081,7 @@
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>YW-BA-017</t>
+          <t>YW-BA-026</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4095,13 +4095,13 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F102" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G102" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -4117,7 +4117,7 @@
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>YW-BA-018</t>
+          <t>YW-BA-027</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4131,13 +4131,13 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F103" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G103" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -4153,7 +4153,7 @@
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>YW-BA-019</t>
+          <t>YW-BA-028</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4167,13 +4167,13 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F104" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G104" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
@@ -4189,7 +4189,7 @@
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>YW-BA-020</t>
+          <t>YW-BA-029</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4203,13 +4203,13 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F105" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="G105" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -4225,7 +4225,7 @@
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>YW-BA-021</t>
+          <t>YW-BA-030</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4239,13 +4239,13 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="F106" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="G106" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
@@ -4261,7 +4261,7 @@
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>YW-BA-022</t>
+          <t>YW-BA-031</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4275,13 +4275,13 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F107" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G107" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
@@ -4297,7 +4297,7 @@
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>YW-BA-023</t>
+          <t>YW-BA-032</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -4311,13 +4311,13 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F108" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G108" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -4333,7 +4333,7 @@
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>YW-BA-024</t>
+          <t>YW-BA-033</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4347,13 +4347,13 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F109" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G109" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
@@ -4369,7 +4369,7 @@
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>YW-BA-025</t>
+          <t>YW-BA-034</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4383,13 +4383,13 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F110" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="G110" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
@@ -4405,7 +4405,7 @@
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>YW-BA-026</t>
+          <t>YW-BA-035</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4419,13 +4419,13 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="F111" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="G111" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
@@ -4441,7 +4441,7 @@
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>YW-BA-027</t>
+          <t>YW-BA-036</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4455,13 +4455,13 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F112" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G112" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>

</xml_diff>